<commit_message>
Add 6 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 43
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-small-businesses.report.xlsx
+++ b/tools/importer/reports/import-small-businesses.report.xlsx
@@ -40,7 +40,7 @@
     <t>au/accountant-bookkeeper-guides.report.json</t>
   </si>
   <si>
-    <t>["hero-split","columns-feature","columns-feature","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry"]</t>
+    <t>["hero-split","columns-feature","columns-feature","cards-features","cards-features","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry"]</t>
   </si>
   <si>
     <t>au/accountant-bookkeeper-guides</t>
@@ -52,7 +52,7 @@
     <t>small-businesses</t>
   </si>
   <si>
-    <t>2026-10-19T03:05:04.059Z</t>
+    <t>2026-10-19T05:47:53.675Z</t>
   </si>
   <si>
     <t>Accountant and Bookkeeper Resources | Xero AU</t>
@@ -64,13 +64,13 @@
     <t>au/accountants-bookkeepers.report.json</t>
   </si>
   <si>
-    <t>["hero-split","columns-feature","columns-feature","columns-feature","cards-features"]</t>
+    <t>["hero-split","columns-feature","columns-feature","columns-feature","cards-features","cards-features","quote-testimonial"]</t>
   </si>
   <si>
     <t>au/accountants-bookkeepers</t>
   </si>
   <si>
-    <t>2026-10-19T03:05:57.084Z</t>
+    <t>2026-10-19T05:47:59.249Z</t>
   </si>
   <si>
     <t>Accounting Practice Management Software | Xero AU</t>
@@ -82,13 +82,13 @@
     <t>au/guides.report.json</t>
   </si>
   <si>
-    <t>["hero-split","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry"]</t>
+    <t>["hero-split","cards-features","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry"]</t>
   </si>
   <si>
     <t>au/guides</t>
   </si>
   <si>
-    <t>2026-10-19T03:08:37.187Z</t>
+    <t>2026-10-19T05:48:14.807Z</t>
   </si>
   <si>
     <t>Small Business Accounting Tips &amp; Guides | Xero AU</t>
@@ -106,7 +106,7 @@
     <t>au/index</t>
   </si>
   <si>
-    <t>2026-10-19T03:14:31.436Z</t>
+    <t>2026-10-19T05:47:48.416Z</t>
   </si>
   <si>
     <t>Software &amp; Solutions for Small Businesses | Xero AU</t>
@@ -124,7 +124,7 @@
     <t>au/integrators</t>
   </si>
   <si>
-    <t>2026-10-19T03:09:31.627Z</t>
+    <t>2026-10-19T05:48:19.416Z</t>
   </si>
   <si>
     <t>Xero Cloud Integrators | Xero AU</t>
@@ -136,13 +136,13 @@
     <t>au/partner-programme.report.json</t>
   </si>
   <si>
-    <t>["hero-split","cards-logos","columns-feature","cards-footnotes","cards-footnotes","cards-footnotes","cards-footnotes","cards-footnotes","cards-footnotes"]</t>
+    <t>["video","hero-split","cards-logos","columns-feature","quote-testimonial","table-comparison","accordion-faq"]</t>
   </si>
   <si>
     <t>au/partner-programme</t>
   </si>
   <si>
-    <t>2026-10-19T03:10:26.008Z</t>
+    <t>2026-10-19T05:48:24.140Z</t>
   </si>
   <si>
     <t>Partner Program | Xero AU</t>
@@ -160,7 +160,7 @@
     <t>au/resources</t>
   </si>
   <si>
-    <t>2026-10-19T03:11:19.912Z</t>
+    <t>2026-10-19T05:48:29.622Z</t>
   </si>
   <si>
     <t>Resources for Doing Business | Xero AU</t>
@@ -172,13 +172,13 @@
     <t>au/accountants-bookkeepers/bookkeepers.report.json</t>
   </si>
   <si>
-    <t>["hero-split","columns-feature","columns-feature","columns-feature","columns-feature","cards-industry"]</t>
+    <t>["hero-split","columns-feature","columns-feature","columns-feature","columns-feature","cards-industry","quote-testimonial"]</t>
   </si>
   <si>
     <t>au/accountants-bookkeepers/bookkeepers</t>
   </si>
   <si>
-    <t>2026-10-19T03:06:50.834Z</t>
+    <t>2026-10-19T05:48:04.501Z</t>
   </si>
   <si>
     <t>Streamline Your Bookkeeping Practice | Xero AU</t>
@@ -196,7 +196,7 @@
     <t>au/campaign/talk-to-sales</t>
   </si>
   <si>
-    <t>2026-10-19T03:07:44.157Z</t>
+    <t>2026-10-19T05:48:09.527Z</t>
   </si>
   <si>
     <t>Talk to sales | Xero AU</t>
@@ -208,13 +208,13 @@
     <t>au/small-businesses/landlords.report.json</t>
   </si>
   <si>
-    <t>["hero-split","columns-feature","columns-feature","columns-feature","columns-feature","tabs-pricing","cards-industry"]</t>
+    <t>["hero-split","columns-feature","columns-feature","columns-feature","columns-feature","tabs-pricing","cards-industry","columns-intro"]</t>
   </si>
   <si>
     <t>au/small-businesses/landlords</t>
   </si>
   <si>
-    <t>2026-10-19T03:12:13.486Z</t>
+    <t>2026-10-19T05:48:35.617Z</t>
   </si>
   <si>
     <t>Landlords Accounting Software | Xero AU</t>
@@ -226,13 +226,13 @@
     <t>au/small-businesses/manufacturing.report.json</t>
   </si>
   <si>
-    <t>["hero-split","columns-feature","columns-feature","columns-feature","tabs-pricing","cards-industry"]</t>
+    <t>["hero-split","columns-feature","columns-feature","columns-feature","cards-features","cards-features","cards-features","tabs-pricing","cards-industry","columns-intro","quote-testimonial"]</t>
   </si>
   <si>
     <t>au/small-businesses/manufacturing</t>
   </si>
   <si>
-    <t>2026-10-19T03:13:07.974Z</t>
+    <t>2026-10-19T05:48:40.658Z</t>
   </si>
   <si>
     <t>Accounting Software for Manufacturers | Xero AU</t>
@@ -244,13 +244,13 @@
     <t>au/small-businesses/self-employed.report.json</t>
   </si>
   <si>
-    <t>["hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","cards-features","tabs-pricing"]</t>
+    <t>["hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","cards-features","cards-features","tabs-pricing","accordion-faq"]</t>
   </si>
   <si>
     <t>au/small-businesses/self-employed</t>
   </si>
   <si>
-    <t>2026-10-19T03:14:01.989Z</t>
+    <t>2026-10-19T05:48:45.436Z</t>
   </si>
   <si>
     <t>Self-Employed Accounting Software in Australia | Xero AU</t>
@@ -265,7 +265,7 @@
     <t>au/small-businesses/xero-for-self-employed</t>
   </si>
   <si>
-    <t>2026-10-19T03:15:27.208Z</t>
+    <t>2026-10-19T05:48:51.878Z</t>
   </si>
   <si>
     <t>https://www.xero.com/au/small-businesses/xero-for-self-employed/</t>
@@ -274,13 +274,13 @@
     <t>au/small-businesses/xero-for-small-business.report.json</t>
   </si>
   <si>
-    <t>["hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","cards-features","tabs-pricing"]</t>
+    <t>["hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","cards-features","cards-features","tabs-pricing","accordion-faq"]</t>
   </si>
   <si>
     <t>au/small-businesses/xero-for-small-business</t>
   </si>
   <si>
-    <t>2026-10-19T03:16:21.714Z</t>
+    <t>2026-10-19T05:48:57.351Z</t>
   </si>
   <si>
     <t>Small Business Accounting Software Australia | Xero AU</t>

</xml_diff>

<commit_message>
Migrate xero.com/au: importer for all 11 templates, oversized SVG handling
- Shared component mapping and import scripts for 10 more templates (61 pages)
- Parsers: video (per-video Wistia ids), hero-split shapes, quote description,
  cards-testimonial, cards-directory, pricing and comparison table variants
- Cleanup: restore __NEXT_DATA__ for parsers, drop crumbs/G2/forms/duplicates,
  map SVGs over 40KB to rasterized PNGs in DA
- Import script generator; page captures excluded from git

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-small-businesses.report.xlsx
+++ b/tools/importer/reports/import-small-businesses.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="461">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,51 @@
     <t>url</t>
   </si>
   <si>
+    <t>au/about.report.json</t>
+  </si>
+  <si>
+    <t>["quote-testimonial","cards-features","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/about</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>accounting-software</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:19:51.856Z</t>
+  </si>
+  <si>
+    <t>About Xero | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/about/</t>
+  </si>
+  <si>
+    <t>au/accessibility.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>au/accessibility</t>
+  </si>
+  <si>
+    <t>accessibility</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:00:59.520Z</t>
+  </si>
+  <si>
+    <t>Xero Digital Accessibility Statement | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accessibility/</t>
+  </si>
+  <si>
     <t>au/accountant-bookkeeper-guides.report.json</t>
   </si>
   <si>
@@ -46,9 +91,6 @@
     <t>au/accountant-bookkeeper-guides</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>small-businesses</t>
   </si>
   <si>
@@ -70,7 +112,7 @@
     <t>au/accountants-bookkeepers</t>
   </si>
   <si>
-    <t>2026-10-19T05:47:59.249Z</t>
+    <t>2026-10-19T09:19:27.438Z</t>
   </si>
   <si>
     <t>Accounting Practice Management Software | Xero AU</t>
@@ -79,6 +121,120 @@
     <t>https://www.xero.com/au/accountants-bookkeepers/</t>
   </si>
   <si>
+    <t>au/accounting-software.report.json</t>
+  </si>
+  <si>
+    <t>["cards-testimonial","accordion-faq","tabs-pricing","cards-industry","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:59:07.565Z</t>
+  </si>
+  <si>
+    <t>Accounting Software for Australian Small Businesses | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/</t>
+  </si>
+  <si>
+    <t>au/advisors.report.json</t>
+  </si>
+  <si>
+    <t>["cards-directory","cards-features","hero-split"]</t>
+  </si>
+  <si>
+    <t>au/advisors</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:59:44.203Z</t>
+  </si>
+  <si>
+    <t>Find a Bookkeeper or Accountant Near You | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/advisors/</t>
+  </si>
+  <si>
+    <t>au/affiliate-program.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","cards-features","hero-split","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/affiliate-program</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:59:48.739Z</t>
+  </si>
+  <si>
+    <t>Become a Xero Affiliate | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/affiliate-program/</t>
+  </si>
+  <si>
+    <t>au/calculators.report.json</t>
+  </si>
+  <si>
+    <t>["cards-features","cards-features","cards-features"]</t>
+  </si>
+  <si>
+    <t>au/calculators</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:00:03.463Z</t>
+  </si>
+  <si>
+    <t>Calculators | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/calculators/</t>
+  </si>
+  <si>
+    <t>au/certifications.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","cards-directory","columns-intro","cards-features","cards-features","cards-features","hero-split"]</t>
+  </si>
+  <si>
+    <t>au/certifications</t>
+  </si>
+  <si>
+    <t>small-businesses-2</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:01:57.679Z</t>
+  </si>
+  <si>
+    <t>Get Xero Certified &amp; Step Up Your Expertise | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/certifications/</t>
+  </si>
+  <si>
+    <t>au/glossary.report.json</t>
+  </si>
+  <si>
+    <t>["cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry","cards-industry"]</t>
+  </si>
+  <si>
+    <t>au/glossary</t>
+  </si>
+  <si>
+    <t>legal</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:03:26.173Z</t>
+  </si>
+  <si>
+    <t>Accounting Glossary | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/glossary/</t>
+  </si>
+  <si>
     <t>au/guides.report.json</t>
   </si>
   <si>
@@ -106,7 +262,7 @@
     <t>au/index</t>
   </si>
   <si>
-    <t>2026-10-19T05:47:48.416Z</t>
+    <t>2026-10-19T09:23:33.243Z</t>
   </si>
   <si>
     <t>Software &amp; Solutions for Small Businesses | Xero AU</t>
@@ -133,6 +289,42 @@
     <t>https://www.xero.com/au/integrators/</t>
   </si>
   <si>
+    <t>au/investors.report.json</t>
+  </si>
+  <si>
+    <t>["columns-intro","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/investors</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:08.665Z</t>
+  </si>
+  <si>
+    <t>Information for Investors | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/investors/</t>
+  </si>
+  <si>
+    <t>au/media.report.json</t>
+  </si>
+  <si>
+    <t>["hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/media</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:17.650Z</t>
+  </si>
+  <si>
+    <t>Media | Media Releases, Contacts &amp; Downloads | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/media/</t>
+  </si>
+  <si>
     <t>au/partner-programme.report.json</t>
   </si>
   <si>
@@ -142,7 +334,7 @@
     <t>au/partner-programme</t>
   </si>
   <si>
-    <t>2026-10-19T05:48:24.140Z</t>
+    <t>2026-10-19T09:19:37.590Z</t>
   </si>
   <si>
     <t>Partner Program | Xero AU</t>
@@ -151,6 +343,24 @@
     <t>https://www.xero.com/au/partner-programme/</t>
   </si>
   <si>
+    <t>au/pricing-plans.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","accordion-faq","table-comparison","tabs-pricing","cards-logos","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/pricing-plans</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:00:13.729Z</t>
+  </si>
+  <si>
+    <t>Pricing Plans | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/pricing-plans/</t>
+  </si>
+  <si>
     <t>au/resources.report.json</t>
   </si>
   <si>
@@ -169,6 +379,210 @@
     <t>https://www.xero.com/au/resources/</t>
   </si>
   <si>
+    <t>au/sitemap.report.json</t>
+  </si>
+  <si>
+    <t>au/sitemap</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:03:41.133Z</t>
+  </si>
+  <si>
+    <t>Sitemap | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/sitemap/</t>
+  </si>
+  <si>
+    <t>au/small-businesses.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","tabs-pricing","cards-industry","cards-industry","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/small-businesses</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:22.749Z</t>
+  </si>
+  <si>
+    <t>Why Choose Xero for Your Small Business | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/small-businesses/</t>
+  </si>
+  <si>
+    <t>au/sustainability.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/sustainability</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:00:29.707Z</t>
+  </si>
+  <si>
+    <t>Sustainability at Xero | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/sustainability/</t>
+  </si>
+  <si>
+    <t>au/syft-from-xero.report.json</t>
+  </si>
+  <si>
+    <t>["video","accordion-faq","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/syft-from-xero</t>
+  </si>
+  <si>
+    <t>resources</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:03:53.445Z</t>
+  </si>
+  <si>
+    <t>Syft Analytics Generates Actionable Insights Faster | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/syft-from-xero/</t>
+  </si>
+  <si>
+    <t>au/templates.report.json</t>
+  </si>
+  <si>
+    <t>["cards-industry"]</t>
+  </si>
+  <si>
+    <t>au/templates</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:00:34.796Z</t>
+  </si>
+  <si>
+    <t>Templates | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/templates/</t>
+  </si>
+  <si>
+    <t>au/xero-ledger-and-cashbook.report.json</t>
+  </si>
+  <si>
+    <t>["video","accordion-faq","cards-industry","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/xero-ledger-and-cashbook</t>
+  </si>
+  <si>
+    <t>xero-ledger-and-cashbook</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:04:06.034Z</t>
+  </si>
+  <si>
+    <t>Ledger &amp; Cashbook Plans for Small Clients | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/xero-ledger-and-cashbook/</t>
+  </si>
+  <si>
+    <t>au/xero-tax.report.json</t>
+  </si>
+  <si>
+    <t>au/xero-tax</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:03:58.496Z</t>
+  </si>
+  <si>
+    <t>Tax Software for BAS &amp; Accounting Firms | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/xero-tax/</t>
+  </si>
+  <si>
+    <t>au/xero-workpapers.report.json</t>
+  </si>
+  <si>
+    <t>["video","accordion-faq","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/xero-workpapers</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:04:10.963Z</t>
+  </si>
+  <si>
+    <t>Workpapers for Accountants | Powered by Xero | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/xero-workpapers/</t>
+  </si>
+  <si>
+    <t>au/about/contact.report.json</t>
+  </si>
+  <si>
+    <t>["hero-split"]</t>
+  </si>
+  <si>
+    <t>au/about/contact</t>
+  </si>
+  <si>
+    <t>about</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:00:52.793Z</t>
+  </si>
+  <si>
+    <t>Contact Us | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/about/contact/</t>
+  </si>
+  <si>
+    <t>au/about/our-brands.report.json</t>
+  </si>
+  <si>
+    <t>["columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/about/our-brands</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:58:52.316Z</t>
+  </si>
+  <si>
+    <t>Our Brands | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/about/our-brands/</t>
+  </si>
+  <si>
+    <t>au/accountants-bookkeepers/accountants.report.json</t>
+  </si>
+  <si>
+    <t>["quote-testimonial","cards-industry","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accountants-bookkeepers/accountants</t>
+  </si>
+  <si>
+    <t>accounting-software-2</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:20:14.986Z</t>
+  </si>
+  <si>
+    <t>Xero AU for Accountants | Collaborate, Report &amp; Grow | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accountants-bookkeepers/accountants/</t>
+  </si>
+  <si>
     <t>au/accountants-bookkeepers/bookkeepers.report.json</t>
   </si>
   <si>
@@ -178,7 +592,7 @@
     <t>au/accountants-bookkeepers/bookkeepers</t>
   </si>
   <si>
-    <t>2026-10-19T05:48:04.501Z</t>
+    <t>2026-10-19T09:23:37.589Z</t>
   </si>
   <si>
     <t>Streamline Your Bookkeeping Practice | Xero AU</t>
@@ -187,6 +601,273 @@
     <t>https://www.xero.com/au/accountants-bookkeepers/bookkeepers/</t>
   </si>
   <si>
+    <t>au/accountants-bookkeepers/enterprise.report.json</t>
+  </si>
+  <si>
+    <t>["quote-testimonial","columns-intro","hero-split","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accountants-bookkeepers/enterprise</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:20:28.451Z</t>
+  </si>
+  <si>
+    <t>Enterprise Accounting Software | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accountants-bookkeepers/enterprise/</t>
+  </si>
+  <si>
+    <t>au/accountants-bookkeepers/partner-hub.report.json</t>
+  </si>
+  <si>
+    <t>["video","quote-testimonial","accordion-faq","accordion-faq","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accountants-bookkeepers/partner-hub</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:20:33.072Z</t>
+  </si>
+  <si>
+    <t>Partner Hub | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accountants-bookkeepers/partner-hub/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/accept-payments.report.json</t>
+  </si>
+  <si>
+    <t>["video","cards-testimonial","accordion-faq","accordion-faq","accordion-faq","tabs-pricing","cards-industry","cards-industry","cards-promo","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/accept-payments</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:01:11.771Z</t>
+  </si>
+  <si>
+    <t>Accept payments online with Xero payment software | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/accept-payments/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/all-features.report.json</t>
+  </si>
+  <si>
+    <t>["quote-testimonial","tabs-pricing","cards-industry","hero-split","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/all-features</t>
+  </si>
+  <si>
+    <t>accounting-software-3</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:20:45.788Z</t>
+  </si>
+  <si>
+    <t>All Xero Features | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/all-features/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/claim-expenses.report.json</t>
+  </si>
+  <si>
+    <t>["video","quote-testimonial","accordion-faq","accordion-faq","tabs-pricing","cards-industry","cards-promo","cards-promo","cards-promo","cards-features","cards-features","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/claim-expenses</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:19:57.544Z</t>
+  </si>
+  <si>
+    <t>Expense Tracking App and Software | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/claim-expenses/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/create-purchase-orders.report.json</t>
+  </si>
+  <si>
+    <t>["cards-testimonial","accordion-faq","tabs-pricing","cards-industry","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/create-purchase-orders</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:59:23.180Z</t>
+  </si>
+  <si>
+    <t>Purchase Order Software for Small Business | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/create-purchase-orders/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/manage-fixed-assets.report.json</t>
+  </si>
+  <si>
+    <t>["video","cards-testimonial","accordion-faq","accordion-faq","tabs-pricing","cards-industry","cards-industry","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/manage-fixed-assets</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:59:27.996Z</t>
+  </si>
+  <si>
+    <t>Manage Your Fixed Assets With Xero | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/manage-fixed-assets/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/manage-inventory.report.json</t>
+  </si>
+  <si>
+    <t>au/accounting-software/manage-inventory</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:01:16.792Z</t>
+  </si>
+  <si>
+    <t>Inventory Management Software | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/manage-inventory/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/pay-bills.report.json</t>
+  </si>
+  <si>
+    <t>["video","cards-testimonial","accordion-faq","accordion-faq","tabs-pricing","cards-industry","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/pay-bills</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:01:43.557Z</t>
+  </si>
+  <si>
+    <t>Accounts Payable Software | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/pay-bills/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/payroll.report.json</t>
+  </si>
+  <si>
+    <t>["video","cards-testimonial","accordion-faq","tabs-pricing","cards-industry","cards-industry","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/payroll</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:59:33.539Z</t>
+  </si>
+  <si>
+    <t>Payroll Software for Australia | STP Compliant | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/payroll/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/send-invoices.report.json</t>
+  </si>
+  <si>
+    <t>["video","cards-testimonial","accordion-faq","tabs-pricing","cards-industry","cards-logos","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/send-invoices</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:01:47.974Z</t>
+  </si>
+  <si>
+    <t>Invoicing Software for Australia | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/send-invoices/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/send-quotes.report.json</t>
+  </si>
+  <si>
+    <t>["video","cards-testimonial","accordion-faq","accordion-faq","tabs-pricing","cards-industry","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/send-quotes</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:01:52.334Z</t>
+  </si>
+  <si>
+    <t>Quotation Software &amp; Online Quotes | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/send-quotes/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/track-projects.report.json</t>
+  </si>
+  <si>
+    <t>["video","cards-testimonial","accordion-faq","tabs-pricing","cards-industry","cards-promo","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/track-projects</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:59:38.861Z</t>
+  </si>
+  <si>
+    <t>Project Tracking Software for Small Business | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/track-projects/</t>
+  </si>
+  <si>
+    <t>au/ai-in-accounting/jax-vision.report.json</t>
+  </si>
+  <si>
+    <t>["video","accordion-faq","tabs-pricing","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/ai-in-accounting/jax-vision</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:59:53.758Z</t>
+  </si>
+  <si>
+    <t>Just Ask Xero | JAX | Your AI Business Companion | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/ai-in-accounting/jax-vision/</t>
+  </si>
+  <si>
+    <t>au/ai-in-accounting/jax.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","tabs-pricing","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/ai-in-accounting/jax</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:59:58.749Z</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/ai-in-accounting/jax/</t>
+  </si>
+  <si>
     <t>au/campaign/talk-to-sales.report.json</t>
   </si>
   <si>
@@ -205,6 +886,198 @@
     <t>https://www.xero.com/au/campaign/talk-to-sales/</t>
   </si>
   <si>
+    <t>au/campaign/xero-partnership.report.json</t>
+  </si>
+  <si>
+    <t>["cards-industry","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/campaign/xero-partnership</t>
+  </si>
+  <si>
+    <t>campaign</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:03:18.689Z</t>
+  </si>
+  <si>
+    <t>Become a Xero Channel Partner | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/campaign/xero-partnership/</t>
+  </si>
+  <si>
+    <t>au/initiative/end-of-financial-year.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","table-comparison","tabs-pricing","cards-industry","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/initiative/end-of-financial-year</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:03.491Z</t>
+  </si>
+  <si>
+    <t>End of Financial Year 2026: EOFY Guide | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/initiative/end-of-financial-year/</t>
+  </si>
+  <si>
+    <t>au/initiative/payday-super.report.json</t>
+  </si>
+  <si>
+    <t>["quote-testimonial","accordion-faq","table-comparison","tabs-pricing","cards-features","cards-features","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/initiative/payday-super</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:20:07.658Z</t>
+  </si>
+  <si>
+    <t>Payday Super: What Employers Need to Know | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/initiative/payday-super/</t>
+  </si>
+  <si>
+    <t>au/investors/governance.report.json</t>
+  </si>
+  <si>
+    <t>au/investors/governance</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:13.143Z</t>
+  </si>
+  <si>
+    <t>Governance | Investor Information | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/investors/governance/</t>
+  </si>
+  <si>
+    <t>au/legal/privacy.report.json</t>
+  </si>
+  <si>
+    <t>au/legal/privacy</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:03:31.081Z</t>
+  </si>
+  <si>
+    <t>Privacy Notice | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/legal/privacy/</t>
+  </si>
+  <si>
+    <t>au/legal/terms.report.json</t>
+  </si>
+  <si>
+    <t>au/legal/terms</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:03:36.464Z</t>
+  </si>
+  <si>
+    <t>Terms of use | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/legal/terms/</t>
+  </si>
+  <si>
+    <t>au/resources/small-business-insights.report.json</t>
+  </si>
+  <si>
+    <t>["video","cards-industry","cards-industry","cards-industry","hero-split"]</t>
+  </si>
+  <si>
+    <t>au/resources/small-business-insights</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:03:48.270Z</t>
+  </si>
+  <si>
+    <t>Xero Small Business Insights | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/resources/small-business-insights/</t>
+  </si>
+  <si>
+    <t>au/small-businesses/construction.report.json</t>
+  </si>
+  <si>
+    <t>["cards-testimonial","accordion-faq","tabs-pricing","cards-industry","cards-features","cards-features","cards-features","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/small-businesses/construction</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:00:19.230Z</t>
+  </si>
+  <si>
+    <t>Construction &amp; Trades Accounting Software | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/small-businesses/construction/</t>
+  </si>
+  <si>
+    <t>au/small-businesses/customers.report.json</t>
+  </si>
+  <si>
+    <t>["tabs-pricing","cards-industry","cards-features"]</t>
+  </si>
+  <si>
+    <t>au/small-businesses/customers</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:28.501Z</t>
+  </si>
+  <si>
+    <t>Customer Stories | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/small-businesses/customers/</t>
+  </si>
+  <si>
+    <t>au/small-businesses/ecommerce.report.json</t>
+  </si>
+  <si>
+    <t>["cards-testimonial","tabs-pricing","cards-industry","columns-intro","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/small-businesses/ecommerce</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:00:24.856Z</t>
+  </si>
+  <si>
+    <t>Accounting for Ecommerce | Ecommerce Bookkeeping Software | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/small-businesses/ecommerce/</t>
+  </si>
+  <si>
+    <t>au/small-businesses/farming.report.json</t>
+  </si>
+  <si>
+    <t>["cards-testimonial","tabs-pricing","cards-industry","columns-intro","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/small-businesses/farming</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:01:21.296Z</t>
+  </si>
+  <si>
+    <t>Farm Accounting Software | Agricultural Accounting | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/small-businesses/farming/</t>
+  </si>
+  <si>
     <t>au/small-businesses/landlords.report.json</t>
   </si>
   <si>
@@ -232,7 +1105,7 @@
     <t>au/small-businesses/manufacturing</t>
   </si>
   <si>
-    <t>2026-10-19T05:48:40.658Z</t>
+    <t>2026-10-19T09:19:42.517Z</t>
   </si>
   <si>
     <t>Accounting Software for Manufacturers | Xero AU</t>
@@ -241,6 +1114,42 @@
     <t>https://www.xero.com/au/small-businesses/manufacturing/</t>
   </si>
   <si>
+    <t>au/small-businesses/non-profit.report.json</t>
+  </si>
+  <si>
+    <t>["quote-testimonial","accordion-faq","tabs-pricing","cards-industry","cards-industry","cards-features","cards-features","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/small-businesses/non-profit</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:20:20.470Z</t>
+  </si>
+  <si>
+    <t>Accounting software for non-profit organisations | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/small-businesses/non-profit/</t>
+  </si>
+  <si>
+    <t>au/small-businesses/real-estate.report.json</t>
+  </si>
+  <si>
+    <t>["quote-testimonial","tabs-pricing","cards-industry","columns-intro","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/small-businesses/real-estate</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:20:38.371Z</t>
+  </si>
+  <si>
+    <t>Real Estate Accounting &amp; Bookkeeping Software | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/small-businesses/real-estate/</t>
+  </si>
+  <si>
     <t>au/small-businesses/self-employed.report.json</t>
   </si>
   <si>
@@ -250,7 +1159,7 @@
     <t>au/small-businesses/self-employed</t>
   </si>
   <si>
-    <t>2026-10-19T05:48:45.436Z</t>
+    <t>2026-10-19T09:23:42.629Z</t>
   </si>
   <si>
     <t>Self-Employed Accounting Software in Australia | Xero AU</t>
@@ -259,13 +1168,31 @@
     <t>https://www.xero.com/au/small-businesses/self-employed/</t>
   </si>
   <si>
+    <t>au/small-businesses/xero-for-medium-sized-business.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","cards-industry","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/small-businesses/xero-for-medium-sized-business</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:39.690Z</t>
+  </si>
+  <si>
+    <t>Accounting Software for Medium-Sized Business AU | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/small-businesses/xero-for-medium-sized-business/</t>
+  </si>
+  <si>
     <t>au/small-businesses/xero-for-self-employed.report.json</t>
   </si>
   <si>
     <t>au/small-businesses/xero-for-self-employed</t>
   </si>
   <si>
-    <t>2026-10-19T05:48:51.878Z</t>
+    <t>2026-10-19T09:23:47.928Z</t>
   </si>
   <si>
     <t>https://www.xero.com/au/small-businesses/xero-for-self-employed/</t>
@@ -287,6 +1214,186 @@
   </si>
   <si>
     <t>https://www.xero.com/au/small-businesses/xero-for-small-business/</t>
+  </si>
+  <si>
+    <t>au/templates/invoice-template.report.json</t>
+  </si>
+  <si>
+    <t>["video","accordion-faq","accordion-faq","accordion-faq","accordion-faq","columns-intro","columns-intro","cards-features","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/templates/invoice-template</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:44.400Z</t>
+  </si>
+  <si>
+    <t>Free Invoice Template – Download a Customisable Invoice Format | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/templates/invoice-template/</t>
+  </si>
+  <si>
+    <t>au/templates/payslip-template.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/templates/payslip-template</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:49.082Z</t>
+  </si>
+  <si>
+    <t>Payslip Template | Free and Fair Work Compliant | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/templates/payslip-template/</t>
+  </si>
+  <si>
+    <t>au/templates/receipt-template.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","cards-industry","columns-intro","cards-features","hero-split","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/templates/receipt-template</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:53.218Z</t>
+  </si>
+  <si>
+    <t>Free Receipt Template Australia | Download Free PDF | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/templates/receipt-template/</t>
+  </si>
+  <si>
+    <t>au/versus/hnry-alternative.report.json</t>
+  </si>
+  <si>
+    <t>["cards-testimonial","table-comparison","tabs-pricing","columns-intro","columns-intro","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/versus/hnry-alternative</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:02:57.828Z</t>
+  </si>
+  <si>
+    <t>Hnry vs Xero | What’s best for your business? | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/versus/hnry-alternative/</t>
+  </si>
+  <si>
+    <t>au/versus/myob-alternative.report.json</t>
+  </si>
+  <si>
+    <t>["cards-testimonial","accordion-faq","table-comparison","tabs-pricing","cards-features","cards-features","cards-features","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/versus/myob-alternative</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:03:03.131Z</t>
+  </si>
+  <si>
+    <t>MYOB vs Xero: Choosing the right software for you | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/versus/myob-alternative/</t>
+  </si>
+  <si>
+    <t>au/versus/quickbooks-alternative.report.json</t>
+  </si>
+  <si>
+    <t>["cards-testimonial","table-comparison","tabs-pricing","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/versus/quickbooks-alternative</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:00:40.084Z</t>
+  </si>
+  <si>
+    <t>A QuickBooks Alternative for Your Small Business | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/versus/quickbooks-alternative/</t>
+  </si>
+  <si>
+    <t>au/versus/reckon-alternative.report.json</t>
+  </si>
+  <si>
+    <t>["cards-testimonial","tabs-pricing","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/versus/reckon-alternative</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:00:45.490Z</t>
+  </si>
+  <si>
+    <t>Reckon vs Xero | A Reckon Alternative | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/versus/reckon-alternative/</t>
+  </si>
+  <si>
+    <t>au/accountants-bookkeepers/partner-hub/practice-management.report.json</t>
+  </si>
+  <si>
+    <t>["video","accordion-faq","accordion-faq","cards-features","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accountants-bookkeepers/partner-hub/practice-management</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:58:57.533Z</t>
+  </si>
+  <si>
+    <t>Practice Management | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accountants-bookkeepers/partner-hub/practice-management/</t>
+  </si>
+  <si>
+    <t>au/accountants-bookkeepers/partner-hub/tax-and-workpapers.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq","accordion-faq","cards-features","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accountants-bookkeepers/partner-hub/tax-and-workpapers</t>
+  </si>
+  <si>
+    <t>2026-10-19T08:59:02.862Z</t>
+  </si>
+  <si>
+    <t>Tax and Workpapers | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accountants-bookkeepers/partner-hub/tax-and-workpapers/</t>
+  </si>
+  <si>
+    <t>au/accounting-software/claim-expenses/track-mileage.report.json</t>
+  </si>
+  <si>
+    <t>["quote-testimonial","accordion-faq","tabs-pricing","cards-industry","cards-promo","cards-features","cards-features","hero-split","columns-feature","columns-feature","columns-feature","columns-feature","columns-feature"]</t>
+  </si>
+  <si>
+    <t>au/accounting-software/claim-expenses/track-mileage</t>
+  </si>
+  <si>
+    <t>2026-10-19T09:20:02.427Z</t>
+  </si>
+  <si>
+    <t>Mileage Tracker | Track &amp; Reimburse Mileage | Xero AU</t>
+  </si>
+  <si>
+    <t>https://www.xero.com/au/accounting-software/claim-expenses/track-mileage/</t>
   </si>
 </sst>
 </file>
@@ -675,13 +1782,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="45" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
+    <col min="5" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -751,79 +1856,79 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
         <v>11</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
         <v>11</v>
@@ -832,24 +1937,24 @@
         <v>12</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -858,24 +1963,24 @@
         <v>12</v>
       </c>
       <c r="F7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -884,24 +1989,24 @@
         <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -910,169 +2015,1755 @@
         <v>12</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>12</v>
+        <v>63</v>
       </c>
       <c r="F10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G10" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H10" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="F11" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G11" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H11" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C12" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F12" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G12" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="H12" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C13" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F13" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G13" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H13" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="C14" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F14" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="G14" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="H14" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="E15" t="s">
+        <v>63</v>
+      </c>
+      <c r="F15" t="s">
+        <v>95</v>
+      </c>
+      <c r="G15" t="s">
+        <v>96</v>
+      </c>
+      <c r="H15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>63</v>
+      </c>
+      <c r="F16" t="s">
+        <v>101</v>
+      </c>
+      <c r="G16" t="s">
+        <v>102</v>
+      </c>
+      <c r="H16" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>104</v>
+      </c>
+      <c r="B17" t="s">
+        <v>105</v>
+      </c>
+      <c r="C17" t="s">
+        <v>106</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" t="s">
+        <v>107</v>
+      </c>
+      <c r="G17" t="s">
+        <v>108</v>
+      </c>
+      <c r="H17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B18" t="s">
+        <v>111</v>
+      </c>
+      <c r="C18" t="s">
+        <v>112</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
         <v>12</v>
       </c>
-      <c r="F15" t="s">
-        <v>89</v>
-      </c>
-      <c r="G15" t="s">
-        <v>90</v>
-      </c>
-      <c r="H15" t="s">
-        <v>91</v>
+      <c r="F18" t="s">
+        <v>113</v>
+      </c>
+      <c r="G18" t="s">
+        <v>114</v>
+      </c>
+      <c r="H18" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" t="s">
+        <v>117</v>
+      </c>
+      <c r="C19" t="s">
+        <v>118</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" t="s">
+        <v>119</v>
+      </c>
+      <c r="G19" t="s">
+        <v>120</v>
+      </c>
+      <c r="H19" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>122</v>
+      </c>
+      <c r="B20" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" t="s">
+        <v>123</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>70</v>
+      </c>
+      <c r="F20" t="s">
+        <v>124</v>
+      </c>
+      <c r="G20" t="s">
+        <v>125</v>
+      </c>
+      <c r="H20" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>127</v>
+      </c>
+      <c r="B21" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21" t="s">
+        <v>129</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>63</v>
+      </c>
+      <c r="F21" t="s">
+        <v>130</v>
+      </c>
+      <c r="G21" t="s">
+        <v>131</v>
+      </c>
+      <c r="H21" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" t="s">
+        <v>135</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" t="s">
+        <v>136</v>
+      </c>
+      <c r="G22" t="s">
+        <v>137</v>
+      </c>
+      <c r="H22" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>139</v>
+      </c>
+      <c r="B23" t="s">
+        <v>140</v>
+      </c>
+      <c r="C23" t="s">
+        <v>141</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>142</v>
+      </c>
+      <c r="F23" t="s">
+        <v>143</v>
+      </c>
+      <c r="G23" t="s">
+        <v>144</v>
+      </c>
+      <c r="H23" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>146</v>
+      </c>
+      <c r="B24" t="s">
+        <v>147</v>
+      </c>
+      <c r="C24" t="s">
+        <v>148</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" t="s">
+        <v>149</v>
+      </c>
+      <c r="G24" t="s">
+        <v>150</v>
+      </c>
+      <c r="H24" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>152</v>
+      </c>
+      <c r="B25" t="s">
+        <v>153</v>
+      </c>
+      <c r="C25" t="s">
+        <v>154</v>
+      </c>
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>155</v>
+      </c>
+      <c r="F25" t="s">
+        <v>156</v>
+      </c>
+      <c r="G25" t="s">
+        <v>157</v>
+      </c>
+      <c r="H25" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B26" t="s">
+        <v>153</v>
+      </c>
+      <c r="C26" t="s">
+        <v>160</v>
+      </c>
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>142</v>
+      </c>
+      <c r="F26" t="s">
+        <v>161</v>
+      </c>
+      <c r="G26" t="s">
+        <v>162</v>
+      </c>
+      <c r="H26" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>164</v>
+      </c>
+      <c r="B27" t="s">
+        <v>165</v>
+      </c>
+      <c r="C27" t="s">
+        <v>166</v>
+      </c>
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>155</v>
+      </c>
+      <c r="F27" t="s">
+        <v>167</v>
+      </c>
+      <c r="G27" t="s">
+        <v>168</v>
+      </c>
+      <c r="H27" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>170</v>
+      </c>
+      <c r="B28" t="s">
+        <v>171</v>
+      </c>
+      <c r="C28" t="s">
+        <v>172</v>
+      </c>
+      <c r="D28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" t="s">
+        <v>173</v>
+      </c>
+      <c r="F28" t="s">
+        <v>174</v>
+      </c>
+      <c r="G28" t="s">
+        <v>175</v>
+      </c>
+      <c r="H28" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>177</v>
+      </c>
+      <c r="B29" t="s">
+        <v>178</v>
+      </c>
+      <c r="C29" t="s">
+        <v>179</v>
+      </c>
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" t="s">
+        <v>180</v>
+      </c>
+      <c r="G29" t="s">
+        <v>181</v>
+      </c>
+      <c r="H29" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>183</v>
+      </c>
+      <c r="B30" t="s">
+        <v>184</v>
+      </c>
+      <c r="C30" t="s">
+        <v>185</v>
+      </c>
+      <c r="D30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>186</v>
+      </c>
+      <c r="F30" t="s">
+        <v>187</v>
+      </c>
+      <c r="G30" t="s">
+        <v>188</v>
+      </c>
+      <c r="H30" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>190</v>
+      </c>
+      <c r="B31" t="s">
+        <v>191</v>
+      </c>
+      <c r="C31" t="s">
+        <v>192</v>
+      </c>
+      <c r="D31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" t="s">
+        <v>26</v>
+      </c>
+      <c r="F31" t="s">
+        <v>193</v>
+      </c>
+      <c r="G31" t="s">
+        <v>194</v>
+      </c>
+      <c r="H31" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>196</v>
+      </c>
+      <c r="B32" t="s">
+        <v>197</v>
+      </c>
+      <c r="C32" t="s">
+        <v>198</v>
+      </c>
+      <c r="D32" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" t="s">
+        <v>63</v>
+      </c>
+      <c r="F32" t="s">
+        <v>199</v>
+      </c>
+      <c r="G32" t="s">
+        <v>200</v>
+      </c>
+      <c r="H32" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>202</v>
+      </c>
+      <c r="B33" t="s">
+        <v>203</v>
+      </c>
+      <c r="C33" t="s">
+        <v>204</v>
+      </c>
+      <c r="D33" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" t="s">
+        <v>63</v>
+      </c>
+      <c r="F33" t="s">
+        <v>205</v>
+      </c>
+      <c r="G33" t="s">
+        <v>206</v>
+      </c>
+      <c r="H33" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>208</v>
+      </c>
+      <c r="B34" t="s">
+        <v>209</v>
+      </c>
+      <c r="C34" t="s">
+        <v>210</v>
+      </c>
+      <c r="D34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>186</v>
+      </c>
+      <c r="F34" t="s">
+        <v>211</v>
+      </c>
+      <c r="G34" t="s">
+        <v>212</v>
+      </c>
+      <c r="H34" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>214</v>
+      </c>
+      <c r="B35" t="s">
+        <v>215</v>
+      </c>
+      <c r="C35" t="s">
+        <v>216</v>
+      </c>
+      <c r="D35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" t="s">
+        <v>217</v>
+      </c>
+      <c r="F35" t="s">
+        <v>218</v>
+      </c>
+      <c r="G35" t="s">
+        <v>219</v>
+      </c>
+      <c r="H35" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>221</v>
+      </c>
+      <c r="B36" t="s">
+        <v>222</v>
+      </c>
+      <c r="C36" t="s">
+        <v>223</v>
+      </c>
+      <c r="D36" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" t="s">
+        <v>12</v>
+      </c>
+      <c r="F36" t="s">
+        <v>224</v>
+      </c>
+      <c r="G36" t="s">
+        <v>225</v>
+      </c>
+      <c r="H36" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>227</v>
+      </c>
+      <c r="B37" t="s">
+        <v>228</v>
+      </c>
+      <c r="C37" t="s">
+        <v>229</v>
+      </c>
+      <c r="D37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37" t="s">
+        <v>230</v>
+      </c>
+      <c r="G37" t="s">
+        <v>231</v>
+      </c>
+      <c r="H37" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>233</v>
+      </c>
+      <c r="B38" t="s">
+        <v>234</v>
+      </c>
+      <c r="C38" t="s">
+        <v>235</v>
+      </c>
+      <c r="D38" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38" t="s">
+        <v>236</v>
+      </c>
+      <c r="G38" t="s">
+        <v>237</v>
+      </c>
+      <c r="H38" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>239</v>
+      </c>
+      <c r="B39" t="s">
+        <v>228</v>
+      </c>
+      <c r="C39" t="s">
+        <v>240</v>
+      </c>
+      <c r="D39" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" t="s">
+        <v>186</v>
+      </c>
+      <c r="F39" t="s">
+        <v>241</v>
+      </c>
+      <c r="G39" t="s">
+        <v>242</v>
+      </c>
+      <c r="H39" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>244</v>
+      </c>
+      <c r="B40" t="s">
+        <v>245</v>
+      </c>
+      <c r="C40" t="s">
+        <v>246</v>
+      </c>
+      <c r="D40" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" t="s">
+        <v>63</v>
+      </c>
+      <c r="F40" t="s">
+        <v>247</v>
+      </c>
+      <c r="G40" t="s">
+        <v>248</v>
+      </c>
+      <c r="H40" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>250</v>
+      </c>
+      <c r="B41" t="s">
+        <v>251</v>
+      </c>
+      <c r="C41" t="s">
+        <v>252</v>
+      </c>
+      <c r="D41" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" t="s">
+        <v>12</v>
+      </c>
+      <c r="F41" t="s">
+        <v>253</v>
+      </c>
+      <c r="G41" t="s">
+        <v>254</v>
+      </c>
+      <c r="H41" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>256</v>
+      </c>
+      <c r="B42" t="s">
+        <v>257</v>
+      </c>
+      <c r="C42" t="s">
+        <v>258</v>
+      </c>
+      <c r="D42" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" t="s">
+        <v>63</v>
+      </c>
+      <c r="F42" t="s">
+        <v>259</v>
+      </c>
+      <c r="G42" t="s">
+        <v>260</v>
+      </c>
+      <c r="H42" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>262</v>
+      </c>
+      <c r="B43" t="s">
+        <v>263</v>
+      </c>
+      <c r="C43" t="s">
+        <v>264</v>
+      </c>
+      <c r="D43" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" t="s">
+        <v>63</v>
+      </c>
+      <c r="F43" t="s">
+        <v>265</v>
+      </c>
+      <c r="G43" t="s">
+        <v>266</v>
+      </c>
+      <c r="H43" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>268</v>
+      </c>
+      <c r="B44" t="s">
+        <v>269</v>
+      </c>
+      <c r="C44" t="s">
+        <v>270</v>
+      </c>
+      <c r="D44" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" t="s">
+        <v>12</v>
+      </c>
+      <c r="F44" t="s">
+        <v>271</v>
+      </c>
+      <c r="G44" t="s">
+        <v>272</v>
+      </c>
+      <c r="H44" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>274</v>
+      </c>
+      <c r="B45" t="s">
+        <v>275</v>
+      </c>
+      <c r="C45" t="s">
+        <v>276</v>
+      </c>
+      <c r="D45" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" t="s">
+        <v>12</v>
+      </c>
+      <c r="F45" t="s">
+        <v>277</v>
+      </c>
+      <c r="G45" t="s">
+        <v>278</v>
+      </c>
+      <c r="H45" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>280</v>
+      </c>
+      <c r="B46" t="s">
+        <v>281</v>
+      </c>
+      <c r="C46" t="s">
+        <v>282</v>
+      </c>
+      <c r="D46" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" t="s">
+        <v>12</v>
+      </c>
+      <c r="F46" t="s">
+        <v>283</v>
+      </c>
+      <c r="G46" t="s">
+        <v>278</v>
+      </c>
+      <c r="H46" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>285</v>
+      </c>
+      <c r="B47" t="s">
+        <v>286</v>
+      </c>
+      <c r="C47" t="s">
+        <v>287</v>
+      </c>
+      <c r="D47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" t="s">
+        <v>26</v>
+      </c>
+      <c r="F47" t="s">
+        <v>288</v>
+      </c>
+      <c r="G47" t="s">
+        <v>289</v>
+      </c>
+      <c r="H47" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>291</v>
+      </c>
+      <c r="B48" t="s">
+        <v>292</v>
+      </c>
+      <c r="C48" t="s">
+        <v>293</v>
+      </c>
+      <c r="D48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" t="s">
+        <v>294</v>
+      </c>
+      <c r="F48" t="s">
+        <v>295</v>
+      </c>
+      <c r="G48" t="s">
+        <v>296</v>
+      </c>
+      <c r="H48" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>298</v>
+      </c>
+      <c r="B49" t="s">
+        <v>299</v>
+      </c>
+      <c r="C49" t="s">
+        <v>300</v>
+      </c>
+      <c r="D49" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" t="s">
+        <v>63</v>
+      </c>
+      <c r="F49" t="s">
+        <v>301</v>
+      </c>
+      <c r="G49" t="s">
+        <v>302</v>
+      </c>
+      <c r="H49" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>304</v>
+      </c>
+      <c r="B50" t="s">
+        <v>305</v>
+      </c>
+      <c r="C50" t="s">
+        <v>306</v>
+      </c>
+      <c r="D50" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" t="s">
+        <v>12</v>
+      </c>
+      <c r="F50" t="s">
+        <v>307</v>
+      </c>
+      <c r="G50" t="s">
+        <v>308</v>
+      </c>
+      <c r="H50" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>310</v>
+      </c>
+      <c r="B51" t="s">
+        <v>17</v>
+      </c>
+      <c r="C51" t="s">
+        <v>311</v>
+      </c>
+      <c r="D51" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" t="s">
+        <v>63</v>
+      </c>
+      <c r="F51" t="s">
+        <v>312</v>
+      </c>
+      <c r="G51" t="s">
+        <v>313</v>
+      </c>
+      <c r="H51" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>315</v>
+      </c>
+      <c r="B52" t="s">
+        <v>17</v>
+      </c>
+      <c r="C52" t="s">
+        <v>316</v>
+      </c>
+      <c r="D52" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
+        <v>70</v>
+      </c>
+      <c r="F52" t="s">
+        <v>317</v>
+      </c>
+      <c r="G52" t="s">
+        <v>318</v>
+      </c>
+      <c r="H52" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>320</v>
+      </c>
+      <c r="B53" t="s">
+        <v>17</v>
+      </c>
+      <c r="C53" t="s">
+        <v>321</v>
+      </c>
+      <c r="D53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" t="s">
+        <v>70</v>
+      </c>
+      <c r="F53" t="s">
+        <v>322</v>
+      </c>
+      <c r="G53" t="s">
+        <v>323</v>
+      </c>
+      <c r="H53" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>325</v>
+      </c>
+      <c r="B54" t="s">
+        <v>326</v>
+      </c>
+      <c r="C54" t="s">
+        <v>327</v>
+      </c>
+      <c r="D54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" t="s">
+        <v>142</v>
+      </c>
+      <c r="F54" t="s">
+        <v>328</v>
+      </c>
+      <c r="G54" t="s">
+        <v>329</v>
+      </c>
+      <c r="H54" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>331</v>
+      </c>
+      <c r="B55" t="s">
+        <v>332</v>
+      </c>
+      <c r="C55" t="s">
+        <v>333</v>
+      </c>
+      <c r="D55" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" t="s">
+        <v>12</v>
+      </c>
+      <c r="F55" t="s">
+        <v>334</v>
+      </c>
+      <c r="G55" t="s">
+        <v>335</v>
+      </c>
+      <c r="H55" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>337</v>
+      </c>
+      <c r="B56" t="s">
+        <v>338</v>
+      </c>
+      <c r="C56" t="s">
+        <v>339</v>
+      </c>
+      <c r="D56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" t="s">
+        <v>63</v>
+      </c>
+      <c r="F56" t="s">
+        <v>340</v>
+      </c>
+      <c r="G56" t="s">
+        <v>341</v>
+      </c>
+      <c r="H56" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>343</v>
+      </c>
+      <c r="B57" t="s">
+        <v>344</v>
+      </c>
+      <c r="C57" t="s">
+        <v>345</v>
+      </c>
+      <c r="D57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" t="s">
+        <v>12</v>
+      </c>
+      <c r="F57" t="s">
+        <v>346</v>
+      </c>
+      <c r="G57" t="s">
+        <v>347</v>
+      </c>
+      <c r="H57" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>349</v>
+      </c>
+      <c r="B58" t="s">
+        <v>350</v>
+      </c>
+      <c r="C58" t="s">
+        <v>351</v>
+      </c>
+      <c r="D58" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" t="s">
+        <v>186</v>
+      </c>
+      <c r="F58" t="s">
+        <v>352</v>
+      </c>
+      <c r="G58" t="s">
+        <v>353</v>
+      </c>
+      <c r="H58" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>355</v>
+      </c>
+      <c r="B59" t="s">
+        <v>356</v>
+      </c>
+      <c r="C59" t="s">
+        <v>357</v>
+      </c>
+      <c r="D59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" t="s">
+        <v>26</v>
+      </c>
+      <c r="F59" t="s">
+        <v>358</v>
+      </c>
+      <c r="G59" t="s">
+        <v>359</v>
+      </c>
+      <c r="H59" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>361</v>
+      </c>
+      <c r="B60" t="s">
+        <v>362</v>
+      </c>
+      <c r="C60" t="s">
+        <v>363</v>
+      </c>
+      <c r="D60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" t="s">
+        <v>26</v>
+      </c>
+      <c r="F60" t="s">
+        <v>364</v>
+      </c>
+      <c r="G60" t="s">
+        <v>365</v>
+      </c>
+      <c r="H60" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>367</v>
+      </c>
+      <c r="B61" t="s">
+        <v>368</v>
+      </c>
+      <c r="C61" t="s">
+        <v>369</v>
+      </c>
+      <c r="D61" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" t="s">
+        <v>186</v>
+      </c>
+      <c r="F61" t="s">
+        <v>370</v>
+      </c>
+      <c r="G61" t="s">
+        <v>371</v>
+      </c>
+      <c r="H61" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>373</v>
+      </c>
+      <c r="B62" t="s">
+        <v>374</v>
+      </c>
+      <c r="C62" t="s">
+        <v>375</v>
+      </c>
+      <c r="D62" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62" t="s">
+        <v>63</v>
+      </c>
+      <c r="F62" t="s">
+        <v>376</v>
+      </c>
+      <c r="G62" t="s">
+        <v>377</v>
+      </c>
+      <c r="H62" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>379</v>
+      </c>
+      <c r="B63" t="s">
+        <v>380</v>
+      </c>
+      <c r="C63" t="s">
+        <v>381</v>
+      </c>
+      <c r="D63" t="s">
+        <v>11</v>
+      </c>
+      <c r="E63" t="s">
+        <v>26</v>
+      </c>
+      <c r="F63" t="s">
+        <v>382</v>
+      </c>
+      <c r="G63" t="s">
+        <v>383</v>
+      </c>
+      <c r="H63" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>385</v>
+      </c>
+      <c r="B64" t="s">
+        <v>386</v>
+      </c>
+      <c r="C64" t="s">
+        <v>387</v>
+      </c>
+      <c r="D64" t="s">
+        <v>11</v>
+      </c>
+      <c r="E64" t="s">
+        <v>63</v>
+      </c>
+      <c r="F64" t="s">
+        <v>388</v>
+      </c>
+      <c r="G64" t="s">
+        <v>389</v>
+      </c>
+      <c r="H64" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>391</v>
+      </c>
+      <c r="B65" t="s">
+        <v>380</v>
+      </c>
+      <c r="C65" t="s">
+        <v>392</v>
+      </c>
+      <c r="D65" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" t="s">
+        <v>26</v>
+      </c>
+      <c r="F65" t="s">
+        <v>393</v>
+      </c>
+      <c r="G65" t="s">
+        <v>383</v>
+      </c>
+      <c r="H65" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>395</v>
+      </c>
+      <c r="B66" t="s">
+        <v>396</v>
+      </c>
+      <c r="C66" t="s">
+        <v>397</v>
+      </c>
+      <c r="D66" t="s">
+        <v>11</v>
+      </c>
+      <c r="E66" t="s">
+        <v>26</v>
+      </c>
+      <c r="F66" t="s">
+        <v>398</v>
+      </c>
+      <c r="G66" t="s">
+        <v>399</v>
+      </c>
+      <c r="H66" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>401</v>
+      </c>
+      <c r="B67" t="s">
+        <v>402</v>
+      </c>
+      <c r="C67" t="s">
+        <v>403</v>
+      </c>
+      <c r="D67" t="s">
+        <v>11</v>
+      </c>
+      <c r="E67" t="s">
+        <v>63</v>
+      </c>
+      <c r="F67" t="s">
+        <v>404</v>
+      </c>
+      <c r="G67" t="s">
+        <v>405</v>
+      </c>
+      <c r="H67" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>407</v>
+      </c>
+      <c r="B68" t="s">
+        <v>408</v>
+      </c>
+      <c r="C68" t="s">
+        <v>409</v>
+      </c>
+      <c r="D68" t="s">
+        <v>11</v>
+      </c>
+      <c r="E68" t="s">
+        <v>63</v>
+      </c>
+      <c r="F68" t="s">
+        <v>410</v>
+      </c>
+      <c r="G68" t="s">
+        <v>411</v>
+      </c>
+      <c r="H68" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>413</v>
+      </c>
+      <c r="B69" t="s">
+        <v>414</v>
+      </c>
+      <c r="C69" t="s">
+        <v>415</v>
+      </c>
+      <c r="D69" t="s">
+        <v>11</v>
+      </c>
+      <c r="E69" t="s">
+        <v>63</v>
+      </c>
+      <c r="F69" t="s">
+        <v>416</v>
+      </c>
+      <c r="G69" t="s">
+        <v>417</v>
+      </c>
+      <c r="H69" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>419</v>
+      </c>
+      <c r="B70" t="s">
+        <v>420</v>
+      </c>
+      <c r="C70" t="s">
+        <v>421</v>
+      </c>
+      <c r="D70" t="s">
+        <v>11</v>
+      </c>
+      <c r="E70" t="s">
+        <v>63</v>
+      </c>
+      <c r="F70" t="s">
+        <v>422</v>
+      </c>
+      <c r="G70" t="s">
+        <v>423</v>
+      </c>
+      <c r="H70" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>425</v>
+      </c>
+      <c r="B71" t="s">
+        <v>426</v>
+      </c>
+      <c r="C71" t="s">
+        <v>427</v>
+      </c>
+      <c r="D71" t="s">
+        <v>11</v>
+      </c>
+      <c r="E71" t="s">
+        <v>63</v>
+      </c>
+      <c r="F71" t="s">
+        <v>428</v>
+      </c>
+      <c r="G71" t="s">
+        <v>429</v>
+      </c>
+      <c r="H71" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>431</v>
+      </c>
+      <c r="B72" t="s">
+        <v>432</v>
+      </c>
+      <c r="C72" t="s">
+        <v>433</v>
+      </c>
+      <c r="D72" t="s">
+        <v>11</v>
+      </c>
+      <c r="E72" t="s">
+        <v>12</v>
+      </c>
+      <c r="F72" t="s">
+        <v>434</v>
+      </c>
+      <c r="G72" t="s">
+        <v>435</v>
+      </c>
+      <c r="H72" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>437</v>
+      </c>
+      <c r="B73" t="s">
+        <v>438</v>
+      </c>
+      <c r="C73" t="s">
+        <v>439</v>
+      </c>
+      <c r="D73" t="s">
+        <v>11</v>
+      </c>
+      <c r="E73" t="s">
+        <v>12</v>
+      </c>
+      <c r="F73" t="s">
+        <v>440</v>
+      </c>
+      <c r="G73" t="s">
+        <v>441</v>
+      </c>
+      <c r="H73" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>443</v>
+      </c>
+      <c r="B74" t="s">
+        <v>444</v>
+      </c>
+      <c r="C74" t="s">
+        <v>445</v>
+      </c>
+      <c r="D74" t="s">
+        <v>11</v>
+      </c>
+      <c r="E74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F74" t="s">
+        <v>446</v>
+      </c>
+      <c r="G74" t="s">
+        <v>447</v>
+      </c>
+      <c r="H74" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>449</v>
+      </c>
+      <c r="B75" t="s">
+        <v>450</v>
+      </c>
+      <c r="C75" t="s">
+        <v>451</v>
+      </c>
+      <c r="D75" t="s">
+        <v>11</v>
+      </c>
+      <c r="E75" t="s">
+        <v>12</v>
+      </c>
+      <c r="F75" t="s">
+        <v>452</v>
+      </c>
+      <c r="G75" t="s">
+        <v>453</v>
+      </c>
+      <c r="H75" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>455</v>
+      </c>
+      <c r="B76" t="s">
+        <v>456</v>
+      </c>
+      <c r="C76" t="s">
+        <v>457</v>
+      </c>
+      <c r="D76" t="s">
+        <v>11</v>
+      </c>
+      <c r="E76" t="s">
+        <v>12</v>
+      </c>
+      <c r="F76" t="s">
+        <v>458</v>
+      </c>
+      <c r="G76" t="s">
+        <v>459</v>
+      </c>
+      <c r="H76" t="s">
+        <v>460</v>
       </c>
     </row>
   </sheetData>

</xml_diff>